<commit_message>
sua file data + phuong
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Hospitals" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Departments" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Doctors" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DoctorSchedules" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hospitals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Departments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Doctors" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DoctorSchedules" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>quan</t>
+          <t>phuong</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -479,24 +479,24 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 1</t>
+          <t>Bệnh viện Tân Định</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>150 Nguyễn Văn Cừ, Quận 1, TP.HCM</t>
+          <t>338 Hai Bà Trưng, Phường Tân Định, TP.HCM</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Quận 1</t>
+          <t>Phường Tân Định</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>10.777789</v>
+        <v>10.7901324</v>
       </c>
       <c r="E2" t="n">
-        <v>106.6905</v>
+        <v>106.6895943</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -526,24 +526,24 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 2</t>
+          <t>Bệnh viện Lê Văn Thịnh</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>289 Hai Bà Trưng, Quận 2, TP.HCM</t>
+          <t>130 Lê Văn Thịnh, Phường Bình Trưng, TP.HCM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Quận 2</t>
+          <t>Phường Bình Trưng</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>10.783464</v>
+        <v>10.782612</v>
       </c>
       <c r="E3" t="n">
-        <v>106.749729</v>
+        <v>106.7691</v>
       </c>
       <c r="F3" t="b">
         <v>0</v>
@@ -573,24 +573,24 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Quận 3</t>
+          <t>Bệnh viện Quận 3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>57 Cách Mạng Tháng 8, Quận 3, TP.HCM</t>
+          <t>114 Trần Quốc Thảo, Phường Xuân Hòa, TP.HCM</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Quận 3</t>
+          <t>Phường Xuân Hòa</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>10.78381</v>
+        <v>10.7847873</v>
       </c>
       <c r="E4" t="n">
-        <v>106.675636</v>
+        <v>106.6839614</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -620,24 +620,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Quận 4</t>
+          <t>Bệnh viện Quận 4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>297 Cách Mạng Tháng 8, Quận 4, TP.HCM</t>
+          <t>63 Bến Vân Đồn, Phường Xóm Chiếu, TP.HCM</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Quận 4</t>
+          <t>Phường Xóm Chiếu</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>10.753653</v>
+        <v>10.7653</v>
       </c>
       <c r="E5" t="n">
-        <v>106.70704</v>
+        <v>106.70218</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -667,24 +667,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Quận 5</t>
+          <t>Bệnh viện Quận 5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>224 Nguyễn Văn Cừ, Quận 5, TP.HCM</t>
+          <t>642A Nguyễn Trãi, Phường Chợ Lớn, TP.HCM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Quận 5</t>
+          <t>Phường Chợ Lớn</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.75932</v>
+        <v>10.754035</v>
       </c>
       <c r="E6" t="n">
-        <v>106.670026</v>
+        <v>106.66581</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -714,24 +714,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Quận 6</t>
+          <t>Bệnh viện Quận 6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>13 Hậu Giang, Quận 6, TP.HCM</t>
+          <t>Đường Chợ Lớn, Phường Bình Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Quận 6</t>
+          <t>Phường Bình Phú</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>10.744984</v>
+        <v>10.7465528</v>
       </c>
       <c r="E7" t="n">
-        <v>106.630564</v>
+        <v>106.6345645</v>
       </c>
       <c r="F7" t="b">
         <v>0</v>
@@ -761,24 +761,24 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Quận 7</t>
+          <t>Bệnh viện Nguyễn Thị Thập</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>184 Trần Hưng Đạo, Quận 7, TP.HCM</t>
+          <t>101 Nguyễn Thị Thập, Phường Tân Mỹ, TP.HCM</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Quận 7</t>
+          <t>Phường Tân Mỹ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>10.740116</v>
+        <v>10.7373313</v>
       </c>
       <c r="E8" t="n">
-        <v>106.724963</v>
+        <v>106.7241657</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
@@ -808,24 +808,24 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Quận 8</t>
+          <t>Bệnh viện Quận 8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>182 Pasteur, Quận 8, TP.HCM</t>
+          <t>82 Cao Lỗ, Phường Chánh Hưng, TP.HCM</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Quận 8</t>
+          <t>Phường Chánh Hưng</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>10.71711</v>
+        <v>10.7416667</v>
       </c>
       <c r="E9" t="n">
-        <v>106.638144</v>
+        <v>106.6763889</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
@@ -855,24 +855,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Quận 9</t>
+          <t>Bệnh viện Lê Văn Việt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>186 Phan Xích Long, Quận 9, TP.HCM</t>
+          <t>387 Lê Văn Việt, Phường Tăng Nhơn Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Quận 9</t>
+          <t>Phường Tăng Nhơn Phú</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10.833855</v>
+        <v>10.8449288</v>
       </c>
       <c r="E10" t="n">
-        <v>106.819934</v>
+        <v>106.7900007</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
@@ -902,24 +902,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Quận 10</t>
+          <t>Bệnh viện Quận 10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>245 Quốc lộ 1A, Quận 10, TP.HCM</t>
+          <t>571 Sư Vạn Hạnh, Phường Hòa Hưng, TP.HCM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Quận 10</t>
+          <t>Phường Hòa Hưng</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10.77129</v>
+        <v>10.7762318</v>
       </c>
       <c r="E11" t="n">
-        <v>106.657869</v>
+        <v>106.6666796</v>
       </c>
       <c r="F11" t="b">
         <v>0</v>
@@ -949,24 +949,24 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 11</t>
+          <t>Bệnh viện Đa khoa Lãnh Binh Thăng</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>50 Quốc lộ 1A, Quận 11, TP.HCM</t>
+          <t>72 Đường Số 5, Phường Bình Thới, TP.HCM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Quận 11</t>
+          <t>Phường Bình Thới</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>10.752497</v>
+        <v>10.760571</v>
       </c>
       <c r="E12" t="n">
-        <v>106.655446</v>
+        <v>106.648121</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -996,24 +996,24 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 12</t>
+          <t>Bệnh viện Trung Mỹ Tây</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>195 Tỉnh lộ 10, Quận 12, TP.HCM</t>
+          <t>111 Đường Thị Mười, Phường Trung Mỹ Tây, TP.HCM</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Quận 12</t>
+          <t>Phường Trung Mỹ Tây</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>10.857864</v>
+        <v>10.860611</v>
       </c>
       <c r="E13" t="n">
-        <v>106.655573</v>
+        <v>106.630781</v>
       </c>
       <c r="F13" t="b">
         <v>0</v>
@@ -1043,24 +1043,24 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Bình Thạnh</t>
+          <t>Bệnh viện Đa khoa Bình Thạnh</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>126 Hậu Giang, Bình Thạnh, TP.HCM</t>
+          <t>132 Lê Văn Duyệt, Phường Gia Định, TP.HCM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bình Thạnh</t>
+          <t>Phường Gia Định</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>10.796846</v>
+        <v>10.7980298</v>
       </c>
       <c r="E14" t="n">
-        <v>106.700391</v>
+        <v>106.6966605</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -1090,24 +1090,24 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Phú Nhuận</t>
+          <t>Bệnh viện Quận Phú Nhuận</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>129 Pasteur, Phú Nhuận, TP.HCM</t>
+          <t>274 Nguyễn Trọng Tuyển, Phường Phú Nhuận, TP.HCM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Phú Nhuận</t>
+          <t>Phường Phú Nhuận</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>10.794788</v>
+        <v>10.798107</v>
       </c>
       <c r="E15" t="n">
-        <v>106.671596</v>
+        <v>106.671822</v>
       </c>
       <c r="F15" t="b">
         <v>0</v>
@@ -1137,24 +1137,24 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Tân Bình</t>
+          <t>Bệnh viện Tân Bình</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>196 Võ Văn Tần, Tân Bình, TP.HCM</t>
+          <t>605 Hoàng Văn Thụ, Phường Tân Sơn Nhất, TP.HCM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tân Bình</t>
+          <t>Phường Tân Sơn Nhất</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>10.798603</v>
+        <v>10.7945055</v>
       </c>
       <c r="E16" t="n">
-        <v>106.651068</v>
+        <v>106.6549856</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -1184,24 +1184,24 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Tân Phú</t>
+          <t>Bệnh viện Quận Tân Phú</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>146 Bạch Đằng, Tân Phú, TP.HCM</t>
+          <t>609-611 Âu Cơ, Phường Tân Phú, TP.HCM</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tân Phú</t>
+          <t>Phường Tân Phú</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>10.787404</v>
+        <v>10.783638</v>
       </c>
       <c r="E17" t="n">
-        <v>106.62119</v>
+        <v>106.6422004</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -1231,24 +1231,24 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Gò Vấp</t>
+          <t>Bệnh viện Gò Vấp</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>97 Quốc lộ 1A, Gò Vấp, TP.HCM</t>
+          <t>641 Thông Tây Hội, Phường Thông Tây Hội, TP.HCM</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Gò Vấp</t>
+          <t>Phường Thông Tây Hội</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>10.846733</v>
+        <v>10.8346486</v>
       </c>
       <c r="E18" t="n">
-        <v>106.667961</v>
+        <v>106.6615499</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -1278,24 +1278,24 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Bình Tân</t>
+          <t>Bệnh viện Bình Tân</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>204 Trần Hưng Đạo, Bình Tân, TP.HCM</t>
+          <t>809 HL2, Phường Bình Trị Đông, TP.HCM</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bình Tân</t>
+          <t>Phường Bình Trị Đông</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>10.769583</v>
+        <v>10.7643601</v>
       </c>
       <c r="E19" t="n">
-        <v>106.603268</v>
+        <v>106.6032103</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
@@ -1325,24 +1325,24 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Thủ Đức</t>
+          <t>Bệnh viện Thành phố Thủ Đức</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>295 Nguyễn Văn Cừ, Thủ Đức, TP.HCM</t>
+          <t>29 Phú Châu, Phường Tam Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Thủ Đức</t>
+          <t>Phường Tam Bình</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>10.86079</v>
+        <v>10.864332</v>
       </c>
       <c r="E20" t="n">
-        <v>106.7608</v>
+        <v>106.745598</v>
       </c>
       <c r="F20" t="b">
         <v>1</v>
@@ -1372,24 +1372,24 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Bình Chánh</t>
+          <t>Bệnh viện Bình Chánh</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>38 Nguyễn Văn Cừ, Bình Chánh, TP.HCM</t>
+          <t>1 Đường Số 1, Khu trung tâm hành chính, Xã Tân Nhựt, TP.HCM</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bình Chánh</t>
+          <t>Xã Tân Nhựt</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>10.708692</v>
+        <v>10.6908806</v>
       </c>
       <c r="E21" t="n">
-        <v>106.625857</v>
+        <v>106.5859827</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
@@ -1419,24 +1419,24 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Hóc Môn</t>
+          <t>Bệnh viện Hóc Môn</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>215 Trần Hưng Đạo, Hóc Môn, TP.HCM</t>
+          <t>79 Bà Triệu, Xã Hóc Môn, TP.HCM</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Hóc Môn</t>
+          <t>Xã Hóc Môn</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>10.895436</v>
+        <v>10.8827069</v>
       </c>
       <c r="E22" t="n">
-        <v>106.598101</v>
+        <v>106.5932745</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -1466,24 +1466,24 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Củ Chi</t>
+          <t>Bệnh viện Củ Chi</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>171 Cách Mạng Tháng 8, Củ Chi, TP.HCM</t>
+          <t>9A Nguyễn Văn Hoài, Xã Tân An Hội, TP.HCM</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Củ Chi</t>
+          <t>Xã Tân An Hội</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>10.964324</v>
+        <v>10.9757269</v>
       </c>
       <c r="E23" t="n">
-        <v>106.501263</v>
+        <v>106.4770729</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -1513,24 +1513,24 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Nhà Bè</t>
+          <t>Bệnh viện Nhà Bè</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>244 Điện Biên Phủ, Nhà Bè, TP.HCM</t>
+          <t>281A Lê Văn Lương, Xã Nhà Bè, TP.HCM</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Nhà Bè</t>
+          <t>Xã Nhà Bè</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>10.698109</v>
+        <v>10.7044461</v>
       </c>
       <c r="E24" t="n">
-        <v>106.729913</v>
+        <v>106.704459</v>
       </c>
       <c r="F24" t="b">
         <v>1</v>
@@ -1565,12 +1565,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>297 Quốc lộ 1A, Cần Giờ, TP.HCM</t>
+          <t>297 Quốc lộ 1A, Xã Cần Giờ, TP.HCM</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Cần Giờ</t>
+          <t>Xã Cần Giờ</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1612,12 +1612,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>214 Lý Thường Kiệt, Quận 1, TP.HCM</t>
+          <t>214 Lý Thường Kiệt, Phường Bến Thành, TP.HCM</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Quận 1</t>
+          <t>Phường Bến Thành</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -1659,12 +1659,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>270 Xa lộ Hà Nội, Quận 2, TP.HCM</t>
+          <t>270 Xa lộ Hà Nội, Phường Bình Trưng, TP.HCM</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Quận 2</t>
+          <t>Phường Bình Trưng</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1706,12 +1706,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>66 Điện Biên Phủ, Quận 3, TP.HCM</t>
+          <t>66 Điện Biên Phủ, Phường Vườn Lài, TP.HCM</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Quận 3</t>
+          <t>Phường Vườn Lài</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1753,12 +1753,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>226 Phan Xích Long, Quận 4, TP.HCM</t>
+          <t>226 Phan Xích Long, Phường Xóm Chiếu, TP.HCM</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Quận 4</t>
+          <t>Phường Xóm Chiếu</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1800,12 +1800,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>249 Kha Vạn Cân, Quận 5, TP.HCM</t>
+          <t>249 Kha Vạn Cân, Phường Chánh Hưng, TP.HCM</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Quận 5</t>
+          <t>Phường Chánh Hưng</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1847,12 +1847,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>15 Trường Sa, Quận 6, TP.HCM</t>
+          <t>15 Trường Sa, Phường Bình Tiên, TP.HCM</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Quận 6</t>
+          <t>Phường Bình Tiên</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1894,12 +1894,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>284 Hậu Giang, Quận 7, TP.HCM</t>
+          <t>284 Hậu Giang, Phường Tân Thuận, TP.HCM</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Quận 7</t>
+          <t>Phường Tân Thuận</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1941,12 +1941,12 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>67 Nguyễn Trãi, Quận 8, TP.HCM</t>
+          <t>67 Nguyễn Trãi, Phường Phú Định, TP.HCM</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Quận 8</t>
+          <t>Phường Phú Định</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1988,12 +1988,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>144 Kha Vạn Cân, Quận 9, TP.HCM</t>
+          <t>144 Kha Vạn Cân, Phường Long Bình, TP.HCM</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Quận 9</t>
+          <t>Phường Long Bình</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -2035,12 +2035,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>64 Hoàng Sa, Quận 10, TP.HCM</t>
+          <t>64 Hoàng Sa, Phường Hòa Hưng, TP.HCM</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Quận 10</t>
+          <t>Phường Hòa Hưng</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -2082,12 +2082,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>111 Điện Biên Phủ, Quận 11, TP.HCM</t>
+          <t>111 Điện Biên Phủ, Phường Minh Phụng, TP.HCM</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Quận 11</t>
+          <t>Phường Minh Phụng</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -2129,12 +2129,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>281 Nguyễn Huệ, Quận 12, TP.HCM</t>
+          <t>281 Nguyễn Huệ, Phường Tân Thới Hiệp, TP.HCM</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Quận 12</t>
+          <t>Phường Tân Thới Hiệp</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -2176,12 +2176,12 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>67 Lý Thường Kiệt, Bình Thạnh, TP.HCM</t>
+          <t>67 Lý Thường Kiệt, Phường Bình Thạnh, TP.HCM</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bình Thạnh</t>
+          <t>Phường Bình Thạnh</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>167 Nguyễn Văn Cừ, Phú Nhuận, TP.HCM</t>
+          <t>167 Nguyễn Văn Cừ, Phường Bình Lợi Trung, TP.HCM</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Phú Nhuận</t>
+          <t>Phường Bình Lợi Trung</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2270,12 +2270,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>50 Hai Bà Trưng, Tân Bình, TP.HCM</t>
+          <t>50 Hai Bà Trưng, Phường Tân Sơn Nhất, TP.HCM</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Tân Bình</t>
+          <t>Phường Tân Sơn Nhất</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2317,12 +2317,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>282 Hậu Giang, Tân Phú, TP.HCM</t>
+          <t>282 Hậu Giang, Phường Tân Sơn Nhì, TP.HCM</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Tân Phú</t>
+          <t>Phường Tân Sơn Nhì</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -2364,12 +2364,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>291 Võ Văn Tần, Gò Vấp, TP.HCM</t>
+          <t>291 Võ Văn Tần, Phường Gò Vấp, TP.HCM</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Gò Vấp</t>
+          <t>Phường Gò Vấp</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -2411,12 +2411,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>226 Cách Mạng Tháng 8, Bình Tân, TP.HCM</t>
+          <t>226 Cách Mạng Tháng 8, Phường Bình Trị Đông, TP.HCM</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Bình Tân</t>
+          <t>Phường Bình Trị Đông</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -2458,12 +2458,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>112 Bạch Đằng, Thủ Đức, TP.HCM</t>
+          <t>112 Bạch Đằng, Phường Linh Xuân, TP.HCM</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Thủ Đức</t>
+          <t>Phường Linh Xuân</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -2505,12 +2505,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>201 Phạm Văn Đồng, Bình Chánh, TP.HCM</t>
+          <t>201 Phạm Văn Đồng, Phường Bình Đông, TP.HCM</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bình Chánh</t>
+          <t>Phường Bình Đông</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -2552,12 +2552,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>136 Nguyễn Văn Cừ, Hóc Môn, TP.HCM</t>
+          <t>136 Nguyễn Văn Cừ, Xã Hóc Môn, TP.HCM</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Hóc Môn</t>
+          <t>Xã Hóc Môn</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -2599,12 +2599,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>293 Nguyễn Văn Cừ, Củ Chi, TP.HCM</t>
+          <t>293 Nguyễn Văn Cừ, Xã Tân An Hội, TP.HCM</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Củ Chi</t>
+          <t>Xã Tân An Hội</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -2646,12 +2646,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>40 Nguyễn Văn Cừ, Nhà Bè, TP.HCM</t>
+          <t>40 Nguyễn Văn Cừ, Xã Nhà Bè, TP.HCM</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Nhà Bè</t>
+          <t>Xã Nhà Bè</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -2693,12 +2693,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>179 Hai Bà Trưng, Cần Giờ, TP.HCM</t>
+          <t>179 Hai Bà Trưng, Xã Cần Giờ, TP.HCM</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Cần Giờ</t>
+          <t>Xã Cần Giờ</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -2740,12 +2740,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>258 Cách Mạng Tháng 8, Quận 1, TP.HCM</t>
+          <t>258 Cách Mạng Tháng 8, Phường Bến Thành, TP.HCM</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Quận 1</t>
+          <t>Phường Bến Thành</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -2787,12 +2787,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>252 Nguyễn Văn Cừ, Quận 2, TP.HCM</t>
+          <t>252 Nguyễn Văn Cừ, Phường Bình Trưng, TP.HCM</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Quận 2</t>
+          <t>Phường Bình Trưng</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 1</t>
+          <t>Bệnh viện Tân Định</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 1</t>
+          <t>Bệnh viện Tân Định</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 2</t>
+          <t>Bệnh viện Lê Văn Thịnh</t>
         </is>
       </c>
     </row>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 2</t>
+          <t>Bệnh viện Lê Văn Thịnh</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Quận 3</t>
+          <t>Bệnh viện Quận 3</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Quận 3</t>
+          <t>Bệnh viện Quận 3</t>
         </is>
       </c>
     </row>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Quận 4</t>
+          <t>Bệnh viện Quận 4</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Quận 4</t>
+          <t>Bệnh viện Quận 4</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Quận 5</t>
+          <t>Bệnh viện Quận 5</t>
         </is>
       </c>
     </row>
@@ -2968,7 +2968,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Quận 5</t>
+          <t>Bệnh viện Quận 5</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Quận 6</t>
+          <t>Bệnh viện Quận 6</t>
         </is>
       </c>
     </row>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Quận 6</t>
+          <t>Bệnh viện Quận 6</t>
         </is>
       </c>
     </row>
@@ -3004,7 +3004,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Quận 7</t>
+          <t>Bệnh viện Nguyễn Thị Thập</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Quận 7</t>
+          <t>Bệnh viện Nguyễn Thị Thập</t>
         </is>
       </c>
     </row>
@@ -3028,7 +3028,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Quận 8</t>
+          <t>Bệnh viện Quận 8</t>
         </is>
       </c>
     </row>
@@ -3040,7 +3040,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Quận 8</t>
+          <t>Bệnh viện Quận 8</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Quận 9</t>
+          <t>Bệnh viện Lê Văn Việt</t>
         </is>
       </c>
     </row>
@@ -3064,7 +3064,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Quận 9</t>
+          <t>Bệnh viện Lê Văn Việt</t>
         </is>
       </c>
     </row>
@@ -3076,7 +3076,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Quận 10</t>
+          <t>Bệnh viện Quận 10</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Quận 10</t>
+          <t>Bệnh viện Quận 10</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 11</t>
+          <t>Bệnh viện Đa khoa Lãnh Binh Thăng</t>
         </is>
       </c>
     </row>
@@ -3112,7 +3112,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 11</t>
+          <t>Bệnh viện Đa khoa Lãnh Binh Thăng</t>
         </is>
       </c>
     </row>
@@ -3124,7 +3124,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 12</t>
+          <t>Bệnh viện Trung Mỹ Tây</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 12</t>
+          <t>Bệnh viện Trung Mỹ Tây</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Bình Thạnh</t>
+          <t>Bệnh viện Đa khoa Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -3160,7 +3160,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Bình Thạnh</t>
+          <t>Bệnh viện Đa khoa Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -3172,7 +3172,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Phú Nhuận</t>
+          <t>Bệnh viện Quận Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Phú Nhuận</t>
+          <t>Bệnh viện Quận Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -3196,7 +3196,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Tân Bình</t>
+          <t>Bệnh viện Tân Bình</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Tân Bình</t>
+          <t>Bệnh viện Tân Bình</t>
         </is>
       </c>
     </row>
@@ -3220,7 +3220,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Tân Phú</t>
+          <t>Bệnh viện Quận Tân Phú</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Tân Phú</t>
+          <t>Bệnh viện Quận Tân Phú</t>
         </is>
       </c>
     </row>
@@ -3244,7 +3244,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Gò Vấp</t>
+          <t>Bệnh viện Gò Vấp</t>
         </is>
       </c>
     </row>
@@ -3256,7 +3256,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Gò Vấp</t>
+          <t>Bệnh viện Gò Vấp</t>
         </is>
       </c>
     </row>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Bình Tân</t>
+          <t>Bệnh viện Bình Tân</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Bình Tân</t>
+          <t>Bệnh viện Bình Tân</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Thủ Đức</t>
+          <t>Bệnh viện Thành phố Thủ Đức</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3304,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Thủ Đức</t>
+          <t>Bệnh viện Thành phố Thủ Đức</t>
         </is>
       </c>
     </row>
@@ -3316,7 +3316,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Bình Chánh</t>
+          <t>Bệnh viện Bình Chánh</t>
         </is>
       </c>
     </row>
@@ -3328,7 +3328,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Bình Chánh</t>
+          <t>Bệnh viện Bình Chánh</t>
         </is>
       </c>
     </row>
@@ -3340,7 +3340,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Hóc Môn</t>
+          <t>Bệnh viện Hóc Môn</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Hóc Môn</t>
+          <t>Bệnh viện Hóc Môn</t>
         </is>
       </c>
     </row>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Củ Chi</t>
+          <t>Bệnh viện Củ Chi</t>
         </is>
       </c>
     </row>
@@ -3376,7 +3376,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Củ Chi</t>
+          <t>Bệnh viện Củ Chi</t>
         </is>
       </c>
     </row>
@@ -3388,7 +3388,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Nhà Bè</t>
+          <t>Bệnh viện Nhà Bè</t>
         </is>
       </c>
     </row>
@@ -3400,7 +3400,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Nhà Bè</t>
+          <t>Bệnh viện Nhà Bè</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 1</t>
+          <t>Bệnh viện Tân Định</t>
         </is>
       </c>
     </row>
@@ -4143,7 +4143,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 1</t>
+          <t>Bệnh viện Tân Định</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 1</t>
+          <t>Bệnh viện Tân Định</t>
         </is>
       </c>
     </row>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 1</t>
+          <t>Bệnh viện Tân Định</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4224,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 2</t>
+          <t>Bệnh viện Lê Văn Thịnh</t>
         </is>
       </c>
     </row>
@@ -4251,7 +4251,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 2</t>
+          <t>Bệnh viện Lê Văn Thịnh</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 2</t>
+          <t>Bệnh viện Lê Văn Thịnh</t>
         </is>
       </c>
     </row>
@@ -4305,7 +4305,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 2</t>
+          <t>Bệnh viện Lê Văn Thịnh</t>
         </is>
       </c>
     </row>
@@ -4332,7 +4332,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Quận 3</t>
+          <t>Bệnh viện Quận 3</t>
         </is>
       </c>
     </row>
@@ -4359,7 +4359,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Quận 3</t>
+          <t>Bệnh viện Quận 3</t>
         </is>
       </c>
     </row>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Quận 3</t>
+          <t>Bệnh viện Quận 3</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Quận 3</t>
+          <t>Bệnh viện Quận 3</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Quận 4</t>
+          <t>Bệnh viện Quận 4</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4467,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Quận 4</t>
+          <t>Bệnh viện Quận 4</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Quận 4</t>
+          <t>Bệnh viện Quận 4</t>
         </is>
       </c>
     </row>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Quận 4</t>
+          <t>Bệnh viện Quận 4</t>
         </is>
       </c>
     </row>
@@ -4548,7 +4548,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Quận 5</t>
+          <t>Bệnh viện Quận 5</t>
         </is>
       </c>
     </row>
@@ -4575,7 +4575,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Quận 5</t>
+          <t>Bệnh viện Quận 5</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Quận 5</t>
+          <t>Bệnh viện Quận 5</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Quận 5</t>
+          <t>Bệnh viện Quận 5</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4656,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Quận 6</t>
+          <t>Bệnh viện Quận 6</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Quận 6</t>
+          <t>Bệnh viện Quận 6</t>
         </is>
       </c>
     </row>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Quận 6</t>
+          <t>Bệnh viện Quận 6</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Quận 6</t>
+          <t>Bệnh viện Quận 6</t>
         </is>
       </c>
     </row>
@@ -4764,7 +4764,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Quận 7</t>
+          <t>Bệnh viện Nguyễn Thị Thập</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Quận 7</t>
+          <t>Bệnh viện Nguyễn Thị Thập</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Quận 7</t>
+          <t>Bệnh viện Nguyễn Thị Thập</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Quận 7</t>
+          <t>Bệnh viện Nguyễn Thị Thập</t>
         </is>
       </c>
     </row>
@@ -4872,7 +4872,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Quận 8</t>
+          <t>Bệnh viện Quận 8</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4899,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Quận 8</t>
+          <t>Bệnh viện Quận 8</t>
         </is>
       </c>
     </row>
@@ -4926,7 +4926,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Quận 8</t>
+          <t>Bệnh viện Quận 8</t>
         </is>
       </c>
     </row>
@@ -4953,7 +4953,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Quận 8</t>
+          <t>Bệnh viện Quận 8</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Quận 9</t>
+          <t>Bệnh viện Lê Văn Việt</t>
         </is>
       </c>
     </row>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Quận 9</t>
+          <t>Bệnh viện Lê Văn Việt</t>
         </is>
       </c>
     </row>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Quận 9</t>
+          <t>Bệnh viện Lê Văn Việt</t>
         </is>
       </c>
     </row>
@@ -5061,7 +5061,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Quận 9</t>
+          <t>Bệnh viện Lê Văn Việt</t>
         </is>
       </c>
     </row>
@@ -5088,7 +5088,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Quận 10</t>
+          <t>Bệnh viện Quận 10</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Quận 10</t>
+          <t>Bệnh viện Quận 10</t>
         </is>
       </c>
     </row>
@@ -5142,7 +5142,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Quận 10</t>
+          <t>Bệnh viện Quận 10</t>
         </is>
       </c>
     </row>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Quận 10</t>
+          <t>Bệnh viện Quận 10</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 11</t>
+          <t>Bệnh viện Đa khoa Lãnh Binh Thăng</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5223,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 11</t>
+          <t>Bệnh viện Đa khoa Lãnh Binh Thăng</t>
         </is>
       </c>
     </row>
@@ -5250,7 +5250,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 11</t>
+          <t>Bệnh viện Đa khoa Lãnh Binh Thăng</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5277,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Quận 11</t>
+          <t>Bệnh viện Đa khoa Lãnh Binh Thăng</t>
         </is>
       </c>
     </row>
@@ -5304,7 +5304,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 12</t>
+          <t>Bệnh viện Trung Mỹ Tây</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 12</t>
+          <t>Bệnh viện Trung Mỹ Tây</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5358,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 12</t>
+          <t>Bệnh viện Trung Mỹ Tây</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5385,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Quận 12</t>
+          <t>Bệnh viện Trung Mỹ Tây</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5412,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Bình Thạnh</t>
+          <t>Bệnh viện Đa khoa Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Bình Thạnh</t>
+          <t>Bệnh viện Đa khoa Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -5466,7 +5466,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Bình Thạnh</t>
+          <t>Bệnh viện Đa khoa Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -5493,7 +5493,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Bình Thạnh</t>
+          <t>Bệnh viện Đa khoa Bình Thạnh</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5520,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Phú Nhuận</t>
+          <t>Bệnh viện Quận Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Phú Nhuận</t>
+          <t>Bệnh viện Quận Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Phú Nhuận</t>
+          <t>Bệnh viện Quận Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5601,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Bệnh viện Quốc tế Phú Nhuận</t>
+          <t>Bệnh viện Quận Phú Nhuận</t>
         </is>
       </c>
     </row>
@@ -5628,7 +5628,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Tân Bình</t>
+          <t>Bệnh viện Tân Bình</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Tân Bình</t>
+          <t>Bệnh viện Tân Bình</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Tân Bình</t>
+          <t>Bệnh viện Tân Bình</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5709,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Bệnh viện Nhi Tân Bình</t>
+          <t>Bệnh viện Tân Bình</t>
         </is>
       </c>
     </row>
@@ -5736,7 +5736,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Tân Phú</t>
+          <t>Bệnh viện Quận Tân Phú</t>
         </is>
       </c>
     </row>
@@ -5763,7 +5763,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Tân Phú</t>
+          <t>Bệnh viện Quận Tân Phú</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5790,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Tân Phú</t>
+          <t>Bệnh viện Quận Tân Phú</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5817,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Bệnh viện Tim Tân Phú</t>
+          <t>Bệnh viện Quận Tân Phú</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Gò Vấp</t>
+          <t>Bệnh viện Gò Vấp</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Gò Vấp</t>
+          <t>Bệnh viện Gò Vấp</t>
         </is>
       </c>
     </row>
@@ -5898,7 +5898,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Gò Vấp</t>
+          <t>Bệnh viện Gò Vấp</t>
         </is>
       </c>
     </row>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Bệnh viện Ung bướu Gò Vấp</t>
+          <t>Bệnh viện Gò Vấp</t>
         </is>
       </c>
     </row>
@@ -5952,7 +5952,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Bình Tân</t>
+          <t>Bệnh viện Bình Tân</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Bình Tân</t>
+          <t>Bệnh viện Bình Tân</t>
         </is>
       </c>
     </row>
@@ -6006,7 +6006,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Bình Tân</t>
+          <t>Bệnh viện Bình Tân</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Bệnh viện Tai Mũi Họng Bình Tân</t>
+          <t>Bệnh viện Bình Tân</t>
         </is>
       </c>
     </row>
@@ -6060,7 +6060,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Thủ Đức</t>
+          <t>Bệnh viện Thành phố Thủ Đức</t>
         </is>
       </c>
     </row>
@@ -6087,7 +6087,7 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Thủ Đức</t>
+          <t>Bệnh viện Thành phố Thủ Đức</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Thủ Đức</t>
+          <t>Bệnh viện Thành phố Thủ Đức</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6141,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Bệnh viện Mắt Thủ Đức</t>
+          <t>Bệnh viện Thành phố Thủ Đức</t>
         </is>
       </c>
     </row>
@@ -6168,7 +6168,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Bình Chánh</t>
+          <t>Bệnh viện Bình Chánh</t>
         </is>
       </c>
     </row>
@@ -6195,7 +6195,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Bình Chánh</t>
+          <t>Bệnh viện Bình Chánh</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6222,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Bình Chánh</t>
+          <t>Bệnh viện Bình Chánh</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6249,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Bệnh viện Sản Bình Chánh</t>
+          <t>Bệnh viện Bình Chánh</t>
         </is>
       </c>
     </row>
@@ -6276,7 +6276,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Hóc Môn</t>
+          <t>Bệnh viện Hóc Môn</t>
         </is>
       </c>
     </row>
@@ -6303,7 +6303,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Hóc Môn</t>
+          <t>Bệnh viện Hóc Môn</t>
         </is>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Hóc Môn</t>
+          <t>Bệnh viện Hóc Môn</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Hóc Môn</t>
+          <t>Bệnh viện Hóc Môn</t>
         </is>
       </c>
     </row>
@@ -6384,7 +6384,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Củ Chi</t>
+          <t>Bệnh viện Củ Chi</t>
         </is>
       </c>
     </row>
@@ -6411,7 +6411,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Củ Chi</t>
+          <t>Bệnh viện Củ Chi</t>
         </is>
       </c>
     </row>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Củ Chi</t>
+          <t>Bệnh viện Củ Chi</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Bệnh viện Chuyên khoa Củ Chi</t>
+          <t>Bệnh viện Củ Chi</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6492,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Nhà Bè</t>
+          <t>Bệnh viện Nhà Bè</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Nhà Bè</t>
+          <t>Bệnh viện Nhà Bè</t>
         </is>
       </c>
     </row>
@@ -6546,7 +6546,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Nhà Bè</t>
+          <t>Bệnh viện Nhà Bè</t>
         </is>
       </c>
     </row>
@@ -6573,7 +6573,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Bệnh viện Tư nhân Nhà Bè</t>
+          <t>Bệnh viện Nhà Bè</t>
         </is>
       </c>
     </row>

</xml_diff>